<commit_message>
fix: al catálogo solo suben los códigos que tienen su ficha
Orden de Darwin: se suben los ENCONTRADOS del Excel, los 120 que tienen su
Word. Los 12 que el maestro lista sin ficha quedan FUERA hasta que Lesly
unifique el código y mande el archivo —un producto sin descripción ni foto no
se puede cotizar—, así que salen del catálogo los 9 que la carga anterior había
dejado activos y no se crea ninguno más.

El catálogo queda en 120 productos, todos con descripción y foto del Word.

Co-Authored-By: Claude Opus 5 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Fichas tecnicas cargadas al CRM - revision 28-08.xlsx
+++ b/docs/Fichas tecnicas cargadas al CRM - revision 28-08.xlsx
@@ -449,7 +449,7 @@
     </row>
     <row r="7">
       <c r="A7" t="str">
-        <v>Del maestro sin ficha: quedan activos, sin descripción ni foto</v>
+        <v>Del maestro sin ficha: quedan FUERA del catálogo</v>
       </c>
       <c r="B7">
         <v>12</v>
@@ -476,7 +476,7 @@
         <v>Productos nuevos</v>
       </c>
       <c r="B11">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="12">
@@ -484,7 +484,7 @@
         <v>Productos retirados</v>
       </c>
       <c r="B12">
-        <v>6</v>
+        <v>15</v>
       </c>
     </row>
     <row r="13">
@@ -492,7 +492,7 @@
         <v>Precios actualizados con el Excel</v>
       </c>
       <c r="B13">
-        <v>14</v>
+        <v>13</v>
       </c>
     </row>
     <row r="15">
@@ -628,7 +628,7 @@
         <v>Falta la ficha</v>
       </c>
       <c r="B32" t="str">
-        <v>los 12 códigos que entraron sin Word</v>
+        <v>los 12 códigos del maestro que no tienen Word</v>
       </c>
     </row>
     <row r="33">
@@ -8582,7 +8582,7 @@
         <v>24999</v>
       </c>
       <c r="O122" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="P122" t="str" xml:space="preserve">
         <v xml:space="preserve">El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»
@@ -8633,7 +8633,7 @@
         <v>950</v>
       </c>
       <c r="O123" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="P123" t="str" xml:space="preserve">
         <v xml:space="preserve">El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»
@@ -8841,7 +8841,7 @@
         <v>14500</v>
       </c>
       <c r="O127" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="P127" t="str" xml:space="preserve">
         <v xml:space="preserve">El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»
@@ -8892,7 +8892,7 @@
         <v>15500</v>
       </c>
       <c r="O128" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="P128" t="str" xml:space="preserve">
         <v xml:space="preserve">El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»
@@ -8943,7 +8943,7 @@
         <v>9300</v>
       </c>
       <c r="O129" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="P129" t="str" xml:space="preserve">
         <v xml:space="preserve">El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»
@@ -8994,7 +8994,7 @@
         <v>9500</v>
       </c>
       <c r="O130" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="P130" t="str" xml:space="preserve">
         <v xml:space="preserve">El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»
@@ -9045,7 +9045,7 @@
         <v>9150</v>
       </c>
       <c r="O131" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="P131" t="str" xml:space="preserve">
         <v xml:space="preserve">El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»
@@ -9096,7 +9096,7 @@
         <v>4500</v>
       </c>
       <c r="O132" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="P132" t="str">
         <v>El maestro lo marca en rojo: «No hay ningun archivo con ese codigo»</v>
@@ -9146,7 +9146,7 @@
         <v>11150</v>
       </c>
       <c r="O133" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="P133" t="str" xml:space="preserve">
         <v xml:space="preserve">El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»
@@ -9162,7 +9162,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E29"/>
+  <dimension ref="A1:E36"/>
   <cols>
     <col min="1" max="1" width="22.83203125" customWidth="1"/>
     <col min="2" max="2" width="12.83203125" customWidth="1"/>
@@ -9202,7 +9202,7 @@
         <v/>
       </c>
       <c r="E2" t="str">
-        <v>Figura en el maestro v2 y no existía en el CRM</v>
+        <v>Figura en el maestro v2 con ficha y no existía en el CRM</v>
       </c>
     </row>
     <row r="3">
@@ -9219,7 +9219,7 @@
         <v/>
       </c>
       <c r="E3" t="str">
-        <v>Figura en el maestro v2 y no existía en el CRM</v>
+        <v>Figura en el maestro v2 con ficha y no existía en el CRM</v>
       </c>
     </row>
     <row r="4">
@@ -9236,7 +9236,7 @@
         <v/>
       </c>
       <c r="E4" t="str">
-        <v>Figura en el maestro v2 y no existía en el CRM</v>
+        <v>Figura en el maestro v2 con ficha y no existía en el CRM</v>
       </c>
     </row>
     <row r="5">
@@ -9253,7 +9253,7 @@
         <v/>
       </c>
       <c r="E5" t="str">
-        <v>Figura en el maestro v2 y no existía en el CRM</v>
+        <v>Figura en el maestro v2 con ficha y no existía en el CRM</v>
       </c>
     </row>
     <row r="6">
@@ -9270,7 +9270,7 @@
         <v/>
       </c>
       <c r="E6" t="str">
-        <v>Figura en el maestro v2 y no existía en el CRM</v>
+        <v>Figura en el maestro v2 con ficha y no existía en el CRM</v>
       </c>
     </row>
     <row r="7">
@@ -9287,7 +9287,7 @@
         <v/>
       </c>
       <c r="E7" t="str">
-        <v>Figura en el maestro v2 y no existía en el CRM</v>
+        <v>Figura en el maestro v2 con ficha y no existía en el CRM</v>
       </c>
     </row>
     <row r="8">
@@ -9304,24 +9304,24 @@
         <v/>
       </c>
       <c r="E8" t="str">
-        <v>Figura en el maestro v2 y no existía en el CRM</v>
+        <v>Figura en el maestro v2 con ficha y no existía en el CRM</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
-        <v>Producto nuevo</v>
+        <v>Precio actualizado</v>
       </c>
       <c r="B9" t="str">
-        <v>LAVA060</v>
+        <v>CALM18</v>
       </c>
       <c r="C9" t="str">
-        <v>LAVADORA INDUSTRIAL</v>
+        <v>MESA DE PLANCHADO ASPIRANTE MOD. FENIX SEMI INDUSTRIAL CON CALDERIN INCORPORADA 1.8 LITROS CALENTAMIENTO ELECTRICO</v>
       </c>
       <c r="D9" t="str">
-        <v/>
+        <v>2250.00</v>
       </c>
       <c r="E9" t="str">
-        <v>Figura en el maestro v2 y no existía en el CRM</v>
+        <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
       </c>
     </row>
     <row r="10">
@@ -9329,13 +9329,13 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B10" t="str">
-        <v>CALM18</v>
+        <v>CALM231</v>
       </c>
       <c r="C10" t="str">
-        <v>MESA DE PLANCHADO ASPIRANTE MOD. FENIX SEMI INDUSTRIAL CON CALDERIN INCORPORADA 1.8 LITROS CALENTAMIENTO ELECTRICO</v>
+        <v>MESA DE PLANCHADO ASPIRANTE MOD. FENIX SEMI INDUSTRIAL CON CALDERIN INCORPORADA 2.3 LITROS CALENTAMIENTO ELECTRICO</v>
       </c>
       <c r="D10" t="str">
-        <v>2250.00</v>
+        <v>2350.00</v>
       </c>
       <c r="E10" t="str">
         <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
@@ -9346,13 +9346,13 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B11" t="str">
-        <v>CALM231</v>
+        <v>CALM4</v>
       </c>
       <c r="C11" t="str">
-        <v>MESA DE PLANCHADO ASPIRANTE MOD. FENIX SEMI INDUSTRIAL CON CALDERIN INCORPORADA 2.3 LITROS CALENTAMIENTO ELECTRICO</v>
+        <v>MESA DE PLANCHADO ASPIRANTE MOD. FENIX SEMI INDUSTRIAL CON CALDERIN INCORPORADA 4 LITROS CALENTAMIENTO ELECTRICO</v>
       </c>
       <c r="D11" t="str">
-        <v>2350.00</v>
+        <v>2500.00</v>
       </c>
       <c r="E11" t="str">
         <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
@@ -9363,13 +9363,13 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B12" t="str">
-        <v>CALM4</v>
+        <v>CO401A</v>
       </c>
       <c r="C12" t="str">
-        <v>MESA DE PLANCHADO ASPIRANTE MOD. FENIX SEMI INDUSTRIAL CON CALDERIN INCORPORADA 4 LITROS CALENTAMIENTO ELECTRICO</v>
+        <v>COCHE UTILITARIO DE PLASTICO MOD. HM-401 Azul</v>
       </c>
       <c r="D12" t="str">
-        <v>2500.00</v>
+        <v>1050.00</v>
       </c>
       <c r="E12" t="str">
         <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
@@ -9380,13 +9380,13 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B13" t="str">
-        <v>CO401A</v>
+        <v>CO402A</v>
       </c>
       <c r="C13" t="str">
-        <v>COCHE UTILITARIO DE PLASTICO MOD. HM-401 Azul</v>
+        <v>CARRO DE LVANDERIA DE PLASTICO MOD. HM-402 Azul</v>
       </c>
       <c r="D13" t="str">
-        <v>1050.00</v>
+        <v>999.00</v>
       </c>
       <c r="E13" t="str">
         <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
@@ -9397,10 +9397,10 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B14" t="str">
-        <v>CO402A</v>
+        <v>CO402B</v>
       </c>
       <c r="C14" t="str">
-        <v>CARRO DE LVANDERIA DE PLASTICO MOD. HM-402 Azul</v>
+        <v>CARRO DE LVANDERIA DE PLASTICO MOD. HM-402 Blanco</v>
       </c>
       <c r="D14" t="str">
         <v>999.00</v>
@@ -9414,10 +9414,10 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B15" t="str">
-        <v>CO402B</v>
+        <v>CO402G</v>
       </c>
       <c r="C15" t="str">
-        <v>CARRO DE LVANDERIA DE PLASTICO MOD. HM-402 Blanco</v>
+        <v>CARRO DE LVANDERIA DE PLASTICO MOD. HM-402 Gris</v>
       </c>
       <c r="D15" t="str">
         <v>999.00</v>
@@ -9431,13 +9431,13 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B16" t="str">
-        <v>CO402G</v>
+        <v>CO408A</v>
       </c>
       <c r="C16" t="str">
-        <v>CARRO DE LVANDERIA DE PLASTICO MOD. HM-402 Gris</v>
+        <v>CARRO DE LVANDERIA DE PLASTICO MOD. HM-408 Azul</v>
       </c>
       <c r="D16" t="str">
-        <v>999.00</v>
+        <v>899.00</v>
       </c>
       <c r="E16" t="str">
         <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
@@ -9448,10 +9448,10 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B17" t="str">
-        <v>CO408A</v>
+        <v>CO408B</v>
       </c>
       <c r="C17" t="str">
-        <v>CARRO DE LVANDERIA DE PLASTICO MOD. HM-408 Azul</v>
+        <v>CARRO DE LVANDERIA DE PLASTICO MOD. HM-408 Blanco</v>
       </c>
       <c r="D17" t="str">
         <v>899.00</v>
@@ -9465,13 +9465,13 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B18" t="str">
-        <v>CO408B</v>
+        <v>LAV040</v>
       </c>
       <c r="C18" t="str">
-        <v>CARRO DE LVANDERIA DE PLASTICO MOD. HM-408 Blanco</v>
+        <v>LAVADORA INDUSTRIAL</v>
       </c>
       <c r="D18" t="str">
-        <v>899.00</v>
+        <v>14500.00</v>
       </c>
       <c r="E18" t="str">
         <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
@@ -9482,13 +9482,13 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B19" t="str">
-        <v>LAV040</v>
+        <v>LAV060</v>
       </c>
       <c r="C19" t="str">
         <v>LAVADORA INDUSTRIAL</v>
       </c>
       <c r="D19" t="str">
-        <v>14500.00</v>
+        <v>16500.00</v>
       </c>
       <c r="E19" t="str">
         <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
@@ -9499,13 +9499,13 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B20" t="str">
-        <v>LAV060</v>
+        <v>SECU752</v>
       </c>
       <c r="C20" t="str">
-        <v>LAVADORA INDUSTRIAL</v>
+        <v>SECADORA INDUSTRIAL</v>
       </c>
       <c r="D20" t="str">
-        <v>16500.00</v>
+        <v>11950.00</v>
       </c>
       <c r="E20" t="str">
         <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
@@ -9516,13 +9516,13 @@
         <v>Precio actualizado</v>
       </c>
       <c r="B21" t="str">
-        <v>LAVA060</v>
+        <v>SECU755</v>
       </c>
       <c r="C21" t="str">
-        <v>LAVADORA INDUSTRIAL</v>
+        <v>SECADORA INDUSTRIAL</v>
       </c>
       <c r="D21" t="str">
-        <v>15500.00</v>
+        <v>9900.00</v>
       </c>
       <c r="E21" t="str">
         <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
@@ -9530,36 +9530,36 @@
     </row>
     <row r="22">
       <c r="A22" t="str">
-        <v>Precio actualizado</v>
+        <v>Retirado del catálogo</v>
       </c>
       <c r="B22" t="str">
-        <v>SECU752</v>
+        <v>1SECU1701</v>
       </c>
       <c r="C22" t="str">
         <v>SECADORA INDUSTRIAL</v>
       </c>
       <c r="D22" t="str">
-        <v>11950.00</v>
+        <v/>
       </c>
       <c r="E22" t="str">
-        <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
+        <v>Está en el maestro pero sin ficha: al sistema solo suben los que tienen su Word</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" t="str">
-        <v>Precio actualizado</v>
+        <v>Retirado del catálogo</v>
       </c>
       <c r="B23" t="str">
-        <v>SECU755</v>
+        <v>CALM23</v>
       </c>
       <c r="C23" t="str">
-        <v>SECADORA INDUSTRIAL</v>
+        <v>CALDERÍN CON PLANCHA</v>
       </c>
       <c r="D23" t="str">
-        <v>9900.00</v>
+        <v/>
       </c>
       <c r="E23" t="str">
-        <v>El libro más nuevo de Lesly (MODIF. UT120 26-08) trae este precio</v>
+        <v>Está en el maestro pero sin ficha: al sistema solo suben los que tienen su Word</v>
       </c>
     </row>
     <row r="24">
@@ -9576,7 +9576,7 @@
         <v/>
       </c>
       <c r="E24" t="str">
-        <v>Su equipo pasó a estar codificado por color (CO401A, CO402A/B/G, CO408A/B)</v>
+        <v>Su equipo ahora está codificado por color (CO401A, CO402A/B/G, CO408A/B)</v>
       </c>
     </row>
     <row r="25">
@@ -9593,7 +9593,7 @@
         <v/>
       </c>
       <c r="E25" t="str">
-        <v>Su equipo pasó a estar codificado por color (CO401A, CO402A/B/G, CO408A/B)</v>
+        <v>Su equipo ahora está codificado por color (CO401A, CO402A/B/G, CO408A/B)</v>
       </c>
     </row>
     <row r="26">
@@ -9610,7 +9610,7 @@
         <v/>
       </c>
       <c r="E26" t="str">
-        <v>Su equipo pasó a estar codificado por color (CO401A, CO402A/B/G, CO408A/B)</v>
+        <v>Su equipo ahora está codificado por color (CO401A, CO402A/B/G, CO408A/B)</v>
       </c>
     </row>
     <row r="27">
@@ -9618,16 +9618,16 @@
         <v>Retirado del catálogo</v>
       </c>
       <c r="B27" t="str">
-        <v>SECU75E</v>
+        <v>LAV135S</v>
       </c>
       <c r="C27" t="str">
-        <v>SECADORA INDUSTRIAL</v>
+        <v>LAVADORA INDUST. FLOT. SOFTWASH</v>
       </c>
       <c r="D27" t="str">
         <v/>
       </c>
       <c r="E27" t="str">
-        <v>El maestro v2 ya no lo lista; el mismo equipo figura con otro código</v>
+        <v>Está en el maestro pero sin ficha: al sistema solo suben los que tienen su Word</v>
       </c>
     </row>
     <row r="28">
@@ -9635,16 +9635,16 @@
         <v>Retirado del catálogo</v>
       </c>
       <c r="B28" t="str">
-        <v>SECU75E2</v>
+        <v>LAVA060</v>
       </c>
       <c r="C28" t="str">
-        <v>SECADORA INDUSTRIAL</v>
+        <v>LAVADORA INDUSTRIAL</v>
       </c>
       <c r="D28" t="str">
         <v/>
       </c>
       <c r="E28" t="str">
-        <v>El maestro v2 ya no lo lista; el mismo equipo figura con otro código</v>
+        <v>Está en el maestro pero sin ficha: al sistema solo suben los que tienen su Word</v>
       </c>
     </row>
     <row r="29">
@@ -9652,7 +9652,7 @@
         <v>Retirado del catálogo</v>
       </c>
       <c r="B29" t="str">
-        <v>SECU75E3</v>
+        <v>SEC75E</v>
       </c>
       <c r="C29" t="str">
         <v>SECADORA INDUSTRIAL</v>
@@ -9661,12 +9661,131 @@
         <v/>
       </c>
       <c r="E29" t="str">
+        <v>Está en el maestro pero sin ficha: al sistema solo suben los que tienen su Word</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="str">
+        <v>Retirado del catálogo</v>
+      </c>
+      <c r="B30" t="str">
+        <v>SEC75E2</v>
+      </c>
+      <c r="C30" t="str">
+        <v>SECADORA INDUSTRIAL</v>
+      </c>
+      <c r="D30" t="str">
+        <v/>
+      </c>
+      <c r="E30" t="str">
+        <v>Está en el maestro pero sin ficha: al sistema solo suben los que tienen su Word</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="str">
+        <v>Retirado del catálogo</v>
+      </c>
+      <c r="B31" t="str">
+        <v>SEC75E3</v>
+      </c>
+      <c r="C31" t="str">
+        <v>SECADORA INDUSTRIAL</v>
+      </c>
+      <c r="D31" t="str">
+        <v/>
+      </c>
+      <c r="E31" t="str">
+        <v>Está en el maestro pero sin ficha: al sistema solo suben los que tienen su Word</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="str">
+        <v>Retirado del catálogo</v>
+      </c>
+      <c r="B32" t="str">
+        <v>SECNSEN</v>
+      </c>
+      <c r="C32" t="str">
+        <v>SECADORA SEMI INDUSTRIAL APILABLE ELÉCTRICA</v>
+      </c>
+      <c r="D32" t="str">
+        <v/>
+      </c>
+      <c r="E32" t="str">
+        <v>Está en el maestro pero sin ficha: al sistema solo suben los que tienen su Word</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="str">
+        <v>Retirado del catálogo</v>
+      </c>
+      <c r="B33" t="str">
+        <v>SECU754</v>
+      </c>
+      <c r="C33" t="str">
+        <v>SECADORA INDUSTRIAL</v>
+      </c>
+      <c r="D33" t="str">
+        <v/>
+      </c>
+      <c r="E33" t="str">
+        <v>Está en el maestro pero sin ficha: al sistema solo suben los que tienen su Word</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="str">
+        <v>Retirado del catálogo</v>
+      </c>
+      <c r="B34" t="str">
+        <v>SECU75E</v>
+      </c>
+      <c r="C34" t="str">
+        <v>SECADORA INDUSTRIAL</v>
+      </c>
+      <c r="D34" t="str">
+        <v/>
+      </c>
+      <c r="E34" t="str">
+        <v>El maestro v2 ya no lo lista; el mismo equipo figura con otro código</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="str">
+        <v>Retirado del catálogo</v>
+      </c>
+      <c r="B35" t="str">
+        <v>SECU75E2</v>
+      </c>
+      <c r="C35" t="str">
+        <v>SECADORA INDUSTRIAL</v>
+      </c>
+      <c r="D35" t="str">
+        <v/>
+      </c>
+      <c r="E35" t="str">
+        <v>El maestro v2 ya no lo lista; el mismo equipo figura con otro código</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="str">
+        <v>Retirado del catálogo</v>
+      </c>
+      <c r="B36" t="str">
+        <v>SECU75E3</v>
+      </c>
+      <c r="C36" t="str">
+        <v>SECADORA INDUSTRIAL</v>
+      </c>
+      <c r="D36" t="str">
+        <v/>
+      </c>
+      <c r="E36" t="str">
         <v>El maestro v2 ya no lo lista; el mismo equipo figura con otro código</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:E29"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E36"/>
   </ignoredErrors>
 </worksheet>
 </file>
@@ -9726,7 +9845,7 @@
         <v>UNIMAC</v>
       </c>
       <c r="D2" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="E2" t="str">
         <v>El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»</v>
@@ -9755,7 +9874,7 @@
         <v>SIMI MONDIAL</v>
       </c>
       <c r="D3" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="E3" t="str">
         <v>El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»</v>
@@ -9871,7 +9990,7 @@
         <v>PRIMUS</v>
       </c>
       <c r="D7" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="E7" t="str">
         <v>El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»</v>
@@ -9900,7 +10019,7 @@
         <v>UNIMAC</v>
       </c>
       <c r="D8" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="E8" t="str">
         <v>El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»</v>
@@ -9929,7 +10048,7 @@
         <v>UNIMAC</v>
       </c>
       <c r="D9" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="E9" t="str">
         <v>El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»</v>
@@ -9958,7 +10077,7 @@
         <v>UNIMAC</v>
       </c>
       <c r="D10" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="E10" t="str">
         <v>El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»</v>
@@ -9987,7 +10106,7 @@
         <v>UNIMAC</v>
       </c>
       <c r="D11" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="E11" t="str">
         <v>El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»</v>
@@ -10016,7 +10135,7 @@
         <v>PRIMUS</v>
       </c>
       <c r="D12" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="E12" t="str">
         <v>El maestro lo marca en rojo: «No hay ningun archivo con ese codigo»</v>
@@ -10045,7 +10164,7 @@
         <v>UNIMAC</v>
       </c>
       <c r="D13" t="str">
-        <v>activo</v>
+        <v>retirado</v>
       </c>
       <c r="E13" t="str">
         <v>El maestro lo marca en rojo: «El archivo existe pero con OTRO codigo»</v>

</xml_diff>